<commit_message>
Wide/long workbook split into three tabs; give chapter 2 its own learning objectives
The wide and long tables now sit on separate sheets with a Start here tab that
explains the difference and links to each. Chapter 1a's objectives no longer
cover chapter 2's material.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165WQeoaB3CPsnpvD7o3Yah
</commit_message>
<xml_diff>
--- a/textbook_examples/mod01_lookup_practice.xlsx
+++ b/textbook_examples/mod01_lookup_practice.xlsx
@@ -2,15 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Lookup" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -30,35 +29,41 @@
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="004A7C59"/>
+      <color rgb="FF4A7C59"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="005C6B62"/>
+      <family val="2"/>
+      <color rgb="FF5C6B62"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="0024302A"/>
+      <family val="2"/>
+      <color rgb="FF24302A"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Consolas"/>
-      <color rgb="002F5D46"/>
+      <family val="2"/>
+      <color rgb="FF2F5D46"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="0024302A"/>
+      <color rgb="FF24302A"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -71,12 +76,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004A7C59"/>
+        <fgColor rgb="FF4A7C59"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F6EFD9"/>
+        <fgColor rgb="FFF6EFD9"/>
       </patternFill>
     </fill>
   </fills>
@@ -92,12 +97,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
@@ -125,10 +127,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -492,299 +499,297 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="3" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" style="14" min="1" max="1"/>
+    <col width="17" customWidth="1" style="14" min="2" max="2"/>
+    <col width="13" customWidth="1" style="14" min="3" max="4"/>
+    <col width="12" customWidth="1" style="14" min="5" max="5"/>
+    <col width="3" customWidth="1" style="14" min="7" max="7"/>
+    <col width="12" customWidth="1" style="14" min="8" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1">
+    <row r="1" ht="18" customHeight="1" s="14">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Looking values up in another table</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="44" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="44" customHeight="1" s="14">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>The prices live in a separate little table (H4:I7), not in the main one.  XLOOKUP finds each field's crop in the price list and brings the price back, so we can work out what the crop is worth.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="18" customHeight="1"/>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="3" ht="18" customHeight="1" s="14"/>
+    <row r="4" ht="18" customHeight="1" s="14">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Crop</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Acres</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Yield (bu/ac)</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Price $/bu</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Crop</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Price $/bu</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+    <row r="5" ht="18" customHeight="1" s="14">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>North</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Canola</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="6" t="n">
         <v>320</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="7" t="n">
         <v>41.2</v>
       </c>
-      <c r="E5" s="9" t="n"/>
-      <c r="G5" s="11" t="inlineStr">
+      <c r="E5" s="8" t="n"/>
+      <c r="G5" s="10" t="inlineStr">
         <is>
           <t>Canola</t>
         </is>
       </c>
-      <c r="H5" s="12" t="n">
+      <c r="H5" s="11" t="n">
         <v>14.2</v>
       </c>
     </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+    <row r="6" ht="18" customHeight="1" s="14">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>South</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Wheat</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="6" t="n">
         <v>250</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="7" t="n">
         <v>58.6</v>
       </c>
-      <c r="E6" s="9" t="n"/>
-      <c r="G6" s="11" t="inlineStr">
+      <c r="E6" s="8" t="n"/>
+      <c r="G6" s="10" t="inlineStr">
         <is>
           <t>Wheat</t>
         </is>
       </c>
-      <c r="H6" s="12" t="n">
+      <c r="H6" s="11" t="n">
         <v>8.35</v>
       </c>
     </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+    <row r="7" ht="18" customHeight="1" s="14">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Creek</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Canola</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="6" t="n">
         <v>180</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="7" t="n">
         <v>37.9</v>
       </c>
-      <c r="E7" s="9" t="n"/>
-      <c r="G7" s="11" t="inlineStr">
+      <c r="E7" s="8" t="n"/>
+      <c r="G7" s="10" t="inlineStr">
         <is>
           <t>Barley</t>
         </is>
       </c>
-      <c r="H7" s="12" t="n">
+      <c r="H7" s="11" t="n">
         <v>5.6</v>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
+    <row r="8" ht="18" customHeight="1" s="14">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Barley</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="6" t="n">
         <v>210</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="7" t="n">
         <v>72.40000000000001</v>
       </c>
-      <c r="E8" s="9" t="n"/>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="E8" s="8" t="n"/>
+    </row>
+    <row r="9" ht="18" customHeight="1" s="14">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Rented</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Wheat</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="6" t="n">
         <v>400</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="7" t="n">
         <v>61.3</v>
       </c>
-      <c r="E9" s="9" t="n"/>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="E9" s="8" t="n"/>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="14">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Airport</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Canola</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="6" t="n">
         <v>150</v>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D10" s="7" t="n">
         <v>44.8</v>
       </c>
-      <c r="E10" s="9" t="n"/>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="E10" s="8" t="n"/>
+    </row>
+    <row r="11" ht="18" customHeight="1" s="14">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Hill</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Barley</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="6" t="n">
         <v>275</v>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="7" t="n">
         <v>68.09999999999999</v>
       </c>
-      <c r="E11" s="9" t="n"/>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="E11" s="8" t="n"/>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="14">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Slough</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Wheat</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="6" t="n">
         <v>330</v>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="D12" s="7" t="n">
         <v>55.2</v>
       </c>
-      <c r="E12" s="9" t="n"/>
-    </row>
-    <row r="13" ht="18" customHeight="1"/>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="E12" s="8" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="14"/>
+    <row r="14" ht="18" customHeight="1" s="14">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>The same lookup, three ways</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="15" ht="18" customHeight="1" s="14">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>XLOOKUP (use this one)</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="10" t="n"/>
-    </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="B15" s="5" t="n"/>
+      <c r="C15" s="15" t="n"/>
+    </row>
+    <row r="16" ht="18" customHeight="1" s="14">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>VLOOKUP (older files)</t>
         </is>
       </c>
-      <c r="B16" s="6" t="n"/>
-      <c r="C16" s="10" t="n"/>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="B16" s="5" t="n"/>
+      <c r="C16" s="15" t="n"/>
+    </row>
+    <row r="17" ht="18" customHeight="1" s="14">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>INDEX/MATCH (older still)</t>
         </is>
       </c>
-      <c r="B17" s="6" t="n"/>
-      <c r="C17" s="10" t="n"/>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="B17" s="5" t="n"/>
+      <c r="C17" s="15" t="n"/>
+    </row>
+    <row r="18" ht="18" customHeight="1" s="14">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>XLOOKUP, crop not in the list</t>
         </is>
       </c>
-      <c r="B18" s="6" t="n"/>
-      <c r="C18" s="10" t="n"/>
-    </row>
-    <row r="19" ht="18" customHeight="1"/>
-    <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="14" t="inlineStr">
+      <c r="B18" s="5" t="n"/>
+      <c r="C18" s="15" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1" s="14"/>
+    <row r="20" ht="32" customHeight="1" s="14">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>All three return the same number.  XLOOKUP is the one to reach for: it takes the column to search and the column to return, it matches exactly by default, and the fourth argument lets you say what to show when nothing is found.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="18" customHeight="1"/>
+    <row r="21" ht="18" customHeight="1" s="14"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A2:F2"/>

</xml_diff>

<commit_message>
Align the lookup section with the edited workbook
The price table moved to A4:B7, so the prose ranges, the example formula, and
the workbook's own intro cell were all pointing at the old H4:I7 location. The
example is now a fenced block rather than loose text with stray $ signs, and
the description matches what the sheet actually shows.

Regenerates the practice twin against the edited workbook.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165WQeoaB3CPsnpvD7o3Yah
</commit_message>
<xml_diff>
--- a/textbook_examples/mod01_lookup_practice.xlsx
+++ b/textbook_examples/mod01_lookup_practice.xlsx
@@ -7,6 +7,7 @@
   </bookViews>
   <sheets>
     <sheet name="Lookup" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -66,6 +67,21 @@
       <color rgb="FF24302A"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF5C6B62"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -97,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -126,13 +142,16 @@
     <xf numFmtId="165" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -498,307 +517,328 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" style="14" min="1" max="1"/>
-    <col width="17" customWidth="1" style="14" min="2" max="2"/>
-    <col width="13" customWidth="1" style="14" min="3" max="4"/>
-    <col width="12" customWidth="1" style="14" min="5" max="5"/>
-    <col width="3" customWidth="1" style="14" min="7" max="7"/>
-    <col width="12" customWidth="1" style="14" min="8" max="9"/>
+    <col width="12" customWidth="1" min="1" max="5"/>
+    <col width="3" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" s="14">
+    <row r="1" ht="18" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Looking values up in another table</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="44" customHeight="1" s="14">
-      <c r="A2" s="13" t="inlineStr">
-        <is>
-          <t>The prices live in a separate little table (H4:I7), not in the main one.  XLOOKUP finds each field's crop in the price list and brings the price back, so we can work out what the crop is worth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1" s="14"/>
-    <row r="4" ht="18" customHeight="1" s="14">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="2" ht="44" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>The prices live in a separate little table (A4:B7), not in the main one.  XLOOKUP finds each field's crop in the price list and brings the price back, so we can work out what the crop is worth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1"/>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Crop</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Price $/bu</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Canola</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>14.2</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>8.35</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Barley</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>5.6</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1"/>
+    <row r="9" ht="18" customHeight="1"/>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Crop</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Acres</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Yield (bu/ac)</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>Price $/bu</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Crop</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Price $/bu</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="18" customHeight="1" s="14">
-      <c r="A5" s="4" t="inlineStr">
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>North</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Canola</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C11" s="6" t="n">
         <v>320</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D11" s="7" t="n">
         <v>41.2</v>
       </c>
-      <c r="E5" s="8" t="n"/>
-      <c r="G5" s="10" t="inlineStr">
+      <c r="E11" s="8" t="n"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Wheat</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>250</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="E12" s="8" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Creek</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Canola</t>
         </is>
       </c>
-      <c r="H5" s="11" t="n">
-        <v>14.2</v>
-      </c>
-    </row>
-    <row r="6" ht="18" customHeight="1" s="14">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>South</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="C13" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="E13" s="8" t="n"/>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Barley</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>210</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>72.40000000000001</v>
+      </c>
+      <c r="E14" s="8" t="n"/>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Rented</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Wheat</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n">
-        <v>250</v>
-      </c>
-      <c r="D6" s="7" t="n">
-        <v>58.6</v>
-      </c>
-      <c r="E6" s="8" t="n"/>
-      <c r="G6" s="10" t="inlineStr">
+      <c r="C15" s="6" t="n">
+        <v>400</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>61.3</v>
+      </c>
+      <c r="E15" s="8" t="n"/>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Airport</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Canola</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>44.8</v>
+      </c>
+      <c r="E16" s="8" t="n"/>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Hill</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Barley</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>275</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>68.09999999999999</v>
+      </c>
+      <c r="E17" s="8" t="n"/>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Slough</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Wheat</t>
         </is>
       </c>
-      <c r="H6" s="11" t="n">
-        <v>8.35</v>
-      </c>
-    </row>
-    <row r="7" ht="18" customHeight="1" s="14">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Creek</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Canola</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>180</v>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>37.9</v>
-      </c>
-      <c r="E7" s="8" t="n"/>
-      <c r="G7" s="10" t="inlineStr">
-        <is>
-          <t>Barley</t>
-        </is>
-      </c>
-      <c r="H7" s="11" t="n">
-        <v>5.6</v>
-      </c>
-    </row>
-    <row r="8" ht="18" customHeight="1" s="14">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Barley</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>210</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>72.40000000000001</v>
-      </c>
-      <c r="E8" s="8" t="n"/>
-    </row>
-    <row r="9" ht="18" customHeight="1" s="14">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Rented</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Wheat</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>400</v>
-      </c>
-      <c r="D9" s="7" t="n">
-        <v>61.3</v>
-      </c>
-      <c r="E9" s="8" t="n"/>
-    </row>
-    <row r="10" ht="18" customHeight="1" s="14">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Airport</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Canola</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="n">
-        <v>150</v>
-      </c>
-      <c r="D10" s="7" t="n">
-        <v>44.8</v>
-      </c>
-      <c r="E10" s="8" t="n"/>
-    </row>
-    <row r="11" ht="18" customHeight="1" s="14">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Hill</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Barley</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="n">
-        <v>275</v>
-      </c>
-      <c r="D11" s="7" t="n">
-        <v>68.09999999999999</v>
-      </c>
-      <c r="E11" s="8" t="n"/>
-    </row>
-    <row r="12" ht="18" customHeight="1" s="14">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Slough</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Wheat</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="n">
+      <c r="C18" s="6" t="n">
         <v>330</v>
       </c>
-      <c r="D12" s="7" t="n">
+      <c r="D18" s="7" t="n">
         <v>55.2</v>
       </c>
-      <c r="E12" s="8" t="n"/>
-    </row>
-    <row r="13" ht="18" customHeight="1" s="14"/>
-    <row r="14" ht="18" customHeight="1" s="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>The same lookup, three ways</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="18" customHeight="1" s="14">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>XLOOKUP (use this one)</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="15" t="n"/>
-    </row>
-    <row r="16" ht="18" customHeight="1" s="14">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>VLOOKUP (older files)</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="15" t="n"/>
-    </row>
-    <row r="17" ht="18" customHeight="1" s="14">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>INDEX/MATCH (older still)</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="15" t="n"/>
-    </row>
-    <row r="18" ht="18" customHeight="1" s="14">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>XLOOKUP, crop not in the list</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="n"/>
-      <c r="C18" s="15" t="n"/>
-    </row>
-    <row r="19" ht="18" customHeight="1" s="14"/>
-    <row r="20" ht="32" customHeight="1" s="14">
-      <c r="A20" s="16" t="inlineStr">
-        <is>
-          <t>All three return the same number.  XLOOKUP is the one to reach for: it takes the column to search and the column to return, it matches exactly by default, and the fourth argument lets you say what to show when nothing is found.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="18" customHeight="1" s="14"/>
+      <c r="E18" s="8" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1"/>
+    <row r="20" ht="36" customHeight="1">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>Note that this is for illustration.  Best practice is to put the two different tables in two different worksheets!</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="13" t="n"/>
+      <c r="B21" s="13" t="n"/>
+      <c r="C21" s="13" t="n"/>
+      <c r="D21" s="13" t="n"/>
+      <c r="E21" s="13" t="n"/>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="13" t="n"/>
+      <c r="B22" s="13" t="n"/>
+      <c r="C22" s="13" t="n"/>
+      <c r="D22" s="13" t="n"/>
+      <c r="E22" s="13" t="n"/>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="13" t="n"/>
+      <c r="B23" s="13" t="n"/>
+      <c r="C23" s="13" t="n"/>
+      <c r="D23" s="13" t="n"/>
+      <c r="E23" s="13" t="n"/>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="13" t="n"/>
+      <c r="B24" s="13" t="n"/>
+      <c r="C24" s="13" t="n"/>
+      <c r="D24" s="13" t="n"/>
+      <c r="E24" s="13" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="13" t="n"/>
+      <c r="B25" s="13" t="n"/>
+      <c r="C25" s="13" t="n"/>
+      <c r="D25" s="13" t="n"/>
+      <c r="E25" s="13" t="n"/>
+    </row>
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" s="13" t="n"/>
+      <c r="B26" s="13" t="n"/>
+      <c r="C26" s="13" t="n"/>
+      <c r="D26" s="13" t="n"/>
+      <c r="E26" s="13" t="n"/>
+    </row>
+    <row r="27" ht="18" customHeight="1"/>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="2">
+    <mergeCell ref="A20:F20"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="C18:F18"/>
-    <mergeCell ref="C17:F17"/>
-    <mergeCell ref="C16:F16"/>
-    <mergeCell ref="C15:F15"/>
-    <mergeCell ref="A20:F20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>